<commit_message>
update superpower workflow sop
</commit_message>
<xml_diff>
--- a/Lifelikegame_Phase_Progress_Tracker_CN.xlsx
+++ b/Lifelikegame_Phase_Progress_Tracker_CN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\limgw\Desktop\studies\lifelikegame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9E1A91-0CC2-45D0-B442-F8658D4B931B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45B6688-13B4-4D97-B3F8-AFC9C8FBCCB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4310,7 +4310,7 @@
         <v>5</v>
       </c>
       <c r="H9" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
feat: centralize backend typed settings
</commit_message>
<xml_diff>
--- a/Lifelikegame_Phase_Progress_Tracker_CN.xlsx
+++ b/Lifelikegame_Phase_Progress_Tracker_CN.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\limgw\Desktop\studies\lifelikegame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45B6688-13B4-4D97-B3F8-AFC9C8FBCCB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AECB17E4-DB1F-4ABA-BF6C-3DF83761C39D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4352,7 +4352,7 @@
         <v>5</v>
       </c>
       <c r="H10" s="4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>8</v>

</xml_diff>